<commit_message>
chore: upload new Domain.xlsx via web UI
</commit_message>
<xml_diff>
--- a/Domain.xlsx
+++ b/Domain.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Results" r:id="rId6" sheetId="2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>126.com</t>
   </si>
@@ -68,15 +67,6 @@
   <si>
     <t>adelaide.edu.au</t>
   </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>FAILED TO LOAD</t>
-  </si>
 </sst>
 </file>
 
@@ -248,7 +238,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="39">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -439,36 +429,6 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="none">
-        <fgColor indexed="42"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="42"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="none">
-        <fgColor indexed="45"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="45"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="none">
-        <fgColor indexed="43"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="43"/>
       </patternFill>
     </fill>
   </fills>
@@ -728,19 +688,13 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="true"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1353,122 +1307,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <cols>
-    <col min="1" max="1" width="46.875" customWidth="true"/>
-    <col min="2" max="2" width="31.25" customWidth="true"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="B1" t="s" s="0">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s" s="6">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s" s="6">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s" s="6">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s" s="6">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s" s="6">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s" s="6">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="0">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s" s="6">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s" s="6">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s" s="6">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s" s="6">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s" s="6">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="B13" t="s" s="6">
-        <v>15</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
 </file>
</xml_diff>